<commit_message>
Tighten ADP alignment scoring with 1/ADP weight and top-10 cap
Switches weight from 1/sqrt(ADP) to 1/ADP and limits the denominator
to the cluster's top 10 ADPs, spreading scores from 58-100 instead of
the previous 62-81 compressed range. Scores capped at 100 to handle
punt-scenario flexibility gains.

https://claude.ai/code/session_01KzrWrtUBwXceoLLfEewo3h
</commit_message>
<xml_diff>
--- a/cluster_adp_alignment_all_scenarios.xlsx
+++ b/cluster_adp_alignment_all_scenarios.xlsx
@@ -75,17 +75,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0084CC16"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0016A34A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EF4444"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0084CC16"/>
       </patternFill>
     </fill>
     <fill>
@@ -149,16 +149,16 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -654,507 +654,507 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="L3" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
         </is>
       </c>
       <c r="N3" s="3" t="n">
         <v>5</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>5T Cards-Jets-Pats-Broncos-Raiders</t>
+          <t>3T Falcons-Bucs-Saints</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="N4" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Mega 7T</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+          <t>5T Cards-Jets-Pats-Broncos-Raiders</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
         </is>
       </c>
       <c r="N5" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3T Chiefs-Chargers-49ers</t>
+          <t>4T Bills-Bears-Packers-Dolphins</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>BAD</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>BAD</t>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>BAD</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M6" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
       <c r="N6" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>73</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>3T Falcons-Bucs-Saints</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+          <t>3T Chiefs-Chargers-49ers</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="K7" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="M7" s="7" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
       <c r="N7" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>4T Ravens-Browns-Colts-Bengals</t>
+          <t>Mega 7T</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>BEST</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="L8" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="M8" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
         </is>
       </c>
       <c r="N8" s="3" t="n">
         <v>5</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>4T Bills-Bears-Packers-Dolphins</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+          <t>4T Ravens-Browns-Colts-Bengals</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
           <t>BEST</t>
         </is>
       </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
+          <t>BAD</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
         </is>
       </c>
       <c r="N9" s="3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1247,62 +1247,62 @@
           <t>3T Falcons-Bucs-Saints</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>OKAY</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
@@ -1311,7 +1311,7 @@
         <v>6</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -1325,57 +1325,57 @@
           <t>OKAY</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
+      <c r="M14" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
@@ -1384,7 +1384,7 @@
         <v>12</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>79</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -1393,62 +1393,62 @@
           <t>4T Ravens-Steelers-Panthers-Bengals</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="L15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
@@ -1457,80 +1457,80 @@
         <v>7</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>78</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Mega 7T</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+          <t>4T Bills-Bears-Packers-Dolphins</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
       <c r="N16" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -1539,17 +1539,17 @@
           <t>3T Chiefs-Chargers-49ers</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>BAD</t>
         </is>
@@ -1559,121 +1559,121 @@
           <t>OKAY</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M17" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
       <c r="N17" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>4T Bills-Bears-Packers-Dolphins</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+          <t>Mega 7T</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
       <c r="N18" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O18" s="3" t="n">
         <v>65</v>
@@ -1685,62 +1685,62 @@
           <t>4T Ravens-Browns-Colts-Bengals</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
@@ -1749,7 +1749,7 @@
         <v>8</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -1842,9 +1842,9 @@
           <t>3T Falcons-Bucs-Saints</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>BAD</t>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -1857,47 +1857,47 @@
           <t>OKAY</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
@@ -1906,7 +1906,7 @@
         <v>6</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24">
@@ -1915,62 +1915,62 @@
           <t>4T Ravens-Steelers-Panthers-Bengals</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="M24" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
@@ -1979,7 +1979,7 @@
         <v>7</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25">
@@ -1988,217 +1988,217 @@
           <t>5T Cards-Jets-Pats-Broncos-Raiders</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="M25" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
       <c r="N25" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Mega 7T</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
+          <t>4T Bills-Bears-Packers-Dolphins</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="M26" s="5" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="M26" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
       <c r="N26" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>3T Chiefs-Chargers-49ers</t>
+          <t>Mega 7T</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>BAD</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>BAD</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>BAD</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="L27" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="M27" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M27" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
       <c r="N27" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>65</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28">
@@ -2207,62 +2207,62 @@
           <t>4T Ravens-Browns-Colts-Bengals</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>OKAY</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="L28" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>GOOD</t>
-        </is>
-      </c>
-      <c r="M28" s="5" t="inlineStr">
+      <c r="M28" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
@@ -2271,80 +2271,80 @@
         <v>8</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>4T Bills-Bears-Packers-Dolphins</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
+          <t>3T Chiefs-Chargers-49ers</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>OKAY</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="K29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="M29" s="5" t="inlineStr">
+      <c r="L29" s="7" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
       <c r="N29" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32">
@@ -2437,7 +2437,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 5 — Score 73</t>
+          <t>No Punt — Best slot 8 — Score 82</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="18" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="E5" s="19" t="inlineStr">
         <is>
-          <t>Kenneth Walker III (16.0), Rashee Rice (16.4)</t>
+          <t>Kenneth Walker III (16.0), Rashee Rice (16.4), Omarion Hampton (18.1)</t>
         </is>
       </c>
     </row>
@@ -2494,60 +2494,60 @@
         <v>2</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Omarion Hampton (RB LAC)</t>
+          <t>Rashee Rice (WR KC)</t>
         </is>
       </c>
       <c r="D6" s="18" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="E6" s="19" t="inlineStr"/>
+        <v>16.4</v>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Kenneth Walker III (16.0), Omarion Hampton (18.1)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="18" t="n">
-        <v>29</v>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>— no fit —</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="19" t="n"/>
+        <v>32</v>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Ladd McConkey (WR LAC)</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="E7" s="19" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="18" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="18" t="n">
-        <v>44</v>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>Ladd McConkey (WR LAC)</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>Mike Evans (54.0)</t>
-        </is>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>— no fit —</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="18" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="18" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="18" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
@@ -2579,7 +2579,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="18" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
@@ -2589,14 +2589,18 @@
       <c r="D11" s="18" t="n">
         <v>84.3</v>
       </c>
-      <c r="E11" s="19" t="inlineStr"/>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Justin Herbert (90.6)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="18" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
@@ -2617,19 +2621,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="18" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Brock Purdy (QB SF)</t>
+          <t>Ricky Pearsall (WR SF)</t>
         </is>
       </c>
       <c r="D13" s="18" t="n">
-        <v>99.7</v>
+        <v>106.8</v>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>George Kittle (96.5), Quentin Johnston (99.2), Ricky Pearsall (106.8)</t>
+          <t>Quentin Johnston (99.2), Brock Purdy (99.7), Travis Kelce (114.7)</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2642,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="18" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
@@ -2659,15 +2663,15 @@
         <v>11</v>
       </c>
       <c r="B15" s="18" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Xavier Worthy (WR KC)</t>
+          <t>Oronde Gadsden II (TE LAC)</t>
         </is>
       </c>
       <c r="D15" s="18" t="n">
-        <v>119.7</v>
+        <v>137.1</v>
       </c>
       <c r="E15" s="19" t="inlineStr"/>
     </row>
@@ -2676,24 +2680,22 @@
         <v>12</v>
       </c>
       <c r="B16" s="18" t="n">
-        <v>140</v>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>Oronde Gadsden II (TE LAC)</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="n">
-        <v>137.1</v>
-      </c>
-      <c r="E16" s="19" t="inlineStr"/>
+        <v>137</v>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>— no fit —</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="18" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="18" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
@@ -2710,7 +2712,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="18" t="n">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
@@ -2727,7 +2729,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
@@ -2748,19 +2750,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="18" t="n">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Emmett Johnson (RB KC)</t>
+          <t>David Njoku (TE LAC)</t>
         </is>
       </c>
       <c r="D20" s="18" t="n">
-        <v>195.4</v>
+        <v>180.5</v>
       </c>
       <c r="E20" s="19" t="inlineStr">
         <is>
-          <t>Tre Harris (199.6)</t>
+          <t>Emmett Johnson (195.4)</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2771,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="18" t="n">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
@@ -2781,7 +2783,7 @@
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>Christian Kirk (202.6), Kimani Vidal (203.0)</t>
+          <t>Emmett Johnson (195.4), Christian Kirk (202.6), Kimani Vidal (203.0)</t>
         </is>
       </c>
     </row>
@@ -2790,39 +2792,45 @@
         <v>18</v>
       </c>
       <c r="B22" s="18" t="n">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>Jake Tonges (TE SF)</t>
+          <t>Kimani Vidal (RB LAC)</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>219.6</v>
-      </c>
-      <c r="E22" s="19" t="inlineStr"/>
+        <v>203</v>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Jake Tonges (219.6)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="18" t="n">
-        <v>221</v>
-      </c>
-      <c r="C23" s="20" t="inlineStr">
-        <is>
-          <t>— no fit —</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
+        <v>224</v>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>Jake Tonges (TE SF)</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>219.6</v>
+      </c>
+      <c r="E23" s="19" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="n">
         <v>20</v>
       </c>
       <c r="B24" s="18" t="n">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
@@ -2835,7 +2843,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 5 — Score 68</t>
+          <t>R1 Punted — Best slot 9 — Score 72</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2879,7 @@
         <v>1</v>
       </c>
       <c r="B29" s="18" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
@@ -2886,60 +2894,60 @@
         <v>2</v>
       </c>
       <c r="B30" s="18" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Omarion Hampton (RB LAC)</t>
+          <t>Kenneth Walker III (RB KC)</t>
         </is>
       </c>
       <c r="D30" s="18" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="E30" s="19" t="inlineStr"/>
+        <v>16</v>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>Rashee Rice (16.4), Omarion Hampton (18.1)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="n">
         <v>3</v>
       </c>
       <c r="B31" s="18" t="n">
-        <v>29</v>
-      </c>
-      <c r="C31" s="20" t="inlineStr">
-        <is>
-          <t>— no fit —</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="19" t="n"/>
+        <v>33</v>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>Ladd McConkey (WR LAC)</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="E31" s="19" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="18" t="n">
         <v>4</v>
       </c>
       <c r="B32" s="18" t="n">
-        <v>44</v>
-      </c>
-      <c r="C32" s="19" t="inlineStr">
-        <is>
-          <t>Ladd McConkey (WR LAC)</t>
-        </is>
-      </c>
-      <c r="D32" s="18" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="E32" s="19" t="inlineStr">
-        <is>
-          <t>Mike Evans (54.0)</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>— no fit —</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="18" t="n">
         <v>5</v>
       </c>
       <c r="B33" s="18" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
@@ -2956,7 +2964,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="18" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
@@ -2971,7 +2979,7 @@
         <v>7</v>
       </c>
       <c r="B35" s="18" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
@@ -2981,14 +2989,18 @@
       <c r="D35" s="18" t="n">
         <v>84.3</v>
       </c>
-      <c r="E35" s="19" t="inlineStr"/>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>Justin Herbert (90.6)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="18" t="n">
         <v>8</v>
       </c>
       <c r="B36" s="18" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
@@ -3009,19 +3021,19 @@
         <v>9</v>
       </c>
       <c r="B37" s="18" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Brock Purdy (QB SF)</t>
+          <t>Ricky Pearsall (WR SF)</t>
         </is>
       </c>
       <c r="D37" s="18" t="n">
-        <v>99.7</v>
+        <v>106.8</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>George Kittle (96.5), Quentin Johnston (99.2), Ricky Pearsall (106.8)</t>
+          <t>Quentin Johnston (99.2), Brock Purdy (99.7), Travis Kelce (114.7)</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3042,7 @@
         <v>10</v>
       </c>
       <c r="B38" s="18" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
@@ -3051,15 +3063,15 @@
         <v>11</v>
       </c>
       <c r="B39" s="18" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Xavier Worthy (WR KC)</t>
+          <t>Oronde Gadsden II (TE LAC)</t>
         </is>
       </c>
       <c r="D39" s="18" t="n">
-        <v>119.7</v>
+        <v>137.1</v>
       </c>
       <c r="E39" s="19" t="inlineStr"/>
     </row>
@@ -3068,24 +3080,22 @@
         <v>12</v>
       </c>
       <c r="B40" s="18" t="n">
-        <v>140</v>
-      </c>
-      <c r="C40" s="19" t="inlineStr">
-        <is>
-          <t>Oronde Gadsden II (TE LAC)</t>
-        </is>
-      </c>
-      <c r="D40" s="18" t="n">
-        <v>137.1</v>
-      </c>
-      <c r="E40" s="19" t="inlineStr"/>
+        <v>136</v>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>— no fit —</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="18" t="n">
         <v>13</v>
       </c>
       <c r="B41" s="18" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
@@ -3102,7 +3112,7 @@
         <v>14</v>
       </c>
       <c r="B42" s="18" t="n">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
@@ -3119,7 +3129,7 @@
         <v>15</v>
       </c>
       <c r="B43" s="18" t="n">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
@@ -3140,19 +3150,19 @@
         <v>16</v>
       </c>
       <c r="B44" s="18" t="n">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Emmett Johnson (RB KC)</t>
+          <t>David Njoku (TE LAC)</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>195.4</v>
+        <v>180.5</v>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>Tre Harris (199.6)</t>
+          <t>Emmett Johnson (195.4)</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3171,7 @@
         <v>17</v>
       </c>
       <c r="B45" s="18" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
@@ -3173,7 +3183,7 @@
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>Christian Kirk (202.6), Kimani Vidal (203.0)</t>
+          <t>Emmett Johnson (195.4), Christian Kirk (202.6), Kimani Vidal (203.0)</t>
         </is>
       </c>
     </row>
@@ -3182,39 +3192,45 @@
         <v>18</v>
       </c>
       <c r="B46" s="18" t="n">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Jake Tonges (TE SF)</t>
+          <t>Kimani Vidal (RB LAC)</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
-        <v>219.6</v>
-      </c>
-      <c r="E46" s="19" t="inlineStr"/>
+        <v>203</v>
+      </c>
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>Christian Kirk (202.6), Jake Tonges (219.6)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="18" t="n">
         <v>19</v>
       </c>
       <c r="B47" s="18" t="n">
-        <v>221</v>
-      </c>
-      <c r="C47" s="20" t="inlineStr">
-        <is>
-          <t>— no fit —</t>
-        </is>
-      </c>
-      <c r="D47" s="19" t="n"/>
-      <c r="E47" s="19" t="n"/>
+        <v>225</v>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>Jake Tonges (TE SF)</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>219.6</v>
+      </c>
+      <c r="E47" s="19" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="18" t="n">
         <v>20</v>
       </c>
       <c r="B48" s="18" t="n">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="C48" s="20" t="inlineStr">
         <is>
@@ -3651,7 +3667,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 2 — Score 73</t>
+          <t>No Punt — Best slot 2 — Score 94</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4061,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 6 — Score 83</t>
+          <t>R1 Punted — Best slot 6 — Score 100</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4473,7 @@
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>R1-R2 Punted — Best slot 6 — Score 81</t>
+          <t>R1-R2 Punted — Best slot 6 — Score 100</t>
         </is>
       </c>
     </row>
@@ -4897,7 +4913,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 9 — Score 69</t>
+          <t>No Punt — Best slot 9 — Score 88</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5321,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 9 — Score 65</t>
+          <t>R1 Punted — Best slot 9 — Score 84</t>
         </is>
       </c>
     </row>
@@ -5707,7 +5723,7 @@
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>R1-R2 Punted — Best slot 7 — Score 62</t>
+          <t>R1-R2 Punted — Best slot 3 — Score 85</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5759,7 @@
         <v>1</v>
       </c>
       <c r="B53" s="18" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C53" s="20" t="inlineStr">
         <is>
@@ -5758,7 +5774,7 @@
         <v>2</v>
       </c>
       <c r="B54" s="18" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C54" s="20" t="inlineStr">
         <is>
@@ -5773,19 +5789,19 @@
         <v>3</v>
       </c>
       <c r="B55" s="18" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Josh Jacobs (RB GB)</t>
+          <t>Josh Allen (QB BUF)</t>
         </is>
       </c>
       <c r="D55" s="18" t="n">
-        <v>29.9</v>
+        <v>24.3</v>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>Colston Loveland (41.9)</t>
+          <t>Josh Jacobs (29.9)</t>
         </is>
       </c>
     </row>
@@ -5794,19 +5810,19 @@
         <v>4</v>
       </c>
       <c r="B56" s="18" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Colston Loveland (TE CHI)</t>
+          <t>DJ Moore (WR BUF)</t>
         </is>
       </c>
       <c r="D56" s="18" t="n">
-        <v>41.9</v>
+        <v>43.8</v>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>DJ Moore (43.8), Luther Burden III (48.4)</t>
+          <t>Luther Burden III (48.4), Rome Odunze (56.7), D'Andre Swift (57.1)</t>
         </is>
       </c>
     </row>
@@ -5815,19 +5831,19 @@
         <v>5</v>
       </c>
       <c r="B57" s="18" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Rome Odunze (WR CHI)</t>
+          <t>Luther Burden III (WR CHI)</t>
         </is>
       </c>
       <c r="D57" s="18" t="n">
-        <v>56.7</v>
+        <v>48.4</v>
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t>D'Andre Swift (57.1), Christian Watson (59.4)</t>
+          <t>Rome Odunze (56.7), D'Andre Swift (57.1), Christian Watson (59.4)</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5852,7 @@
         <v>6</v>
       </c>
       <c r="B58" s="18" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
@@ -5857,7 +5873,7 @@
         <v>7</v>
       </c>
       <c r="B59" s="18" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
@@ -5874,7 +5890,7 @@
         <v>8</v>
       </c>
       <c r="B60" s="18" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
@@ -5895,7 +5911,7 @@
         <v>9</v>
       </c>
       <c r="B61" s="18" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
@@ -5907,7 +5923,7 @@
       </c>
       <c r="E61" s="19" t="inlineStr">
         <is>
-          <t>Jordan Love (109.5), Dalton Kincaid (110.2), Matthew Golden (114.1)</t>
+          <t>Jordan Love (109.5), Dalton Kincaid (110.2)</t>
         </is>
       </c>
     </row>
@@ -5916,7 +5932,7 @@
         <v>10</v>
       </c>
       <c r="B62" s="18" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
@@ -5928,7 +5944,7 @@
       </c>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>Jordan Love (109.5), Dalton Kincaid (110.2), Khalil Shakir (122.1)</t>
+          <t>Khalil Shakir (122.1), Malik Willis (128.9)</t>
         </is>
       </c>
     </row>
@@ -5937,19 +5953,19 @@
         <v>11</v>
       </c>
       <c r="B63" s="18" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Malik Willis (QB MIA)</t>
+          <t>Khalil Shakir (WR BUF)</t>
         </is>
       </c>
       <c r="D63" s="18" t="n">
-        <v>128.9</v>
+        <v>122.1</v>
       </c>
       <c r="E63" s="19" t="inlineStr">
         <is>
-          <t>Khalil Shakir (122.1)</t>
+          <t>Malik Willis (128.9)</t>
         </is>
       </c>
     </row>
@@ -5958,7 +5974,7 @@
         <v>12</v>
       </c>
       <c r="B64" s="18" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
@@ -5973,7 +5989,7 @@
         <v>13</v>
       </c>
       <c r="B65" s="18" t="n">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C65" s="20" t="inlineStr">
         <is>
@@ -5988,7 +6004,7 @@
         <v>14</v>
       </c>
       <c r="B66" s="18" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C66" s="20" t="inlineStr">
         <is>
@@ -6003,7 +6019,7 @@
         <v>15</v>
       </c>
       <c r="B67" s="18" t="n">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
@@ -6020,7 +6036,7 @@
         <v>16</v>
       </c>
       <c r="B68" s="18" t="n">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C68" s="20" t="inlineStr">
         <is>
@@ -6035,7 +6051,7 @@
         <v>17</v>
       </c>
       <c r="B69" s="18" t="n">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C69" s="20" t="inlineStr">
         <is>
@@ -6050,7 +6066,7 @@
         <v>18</v>
       </c>
       <c r="B70" s="18" t="n">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
@@ -6067,7 +6083,7 @@
         <v>19</v>
       </c>
       <c r="B71" s="18" t="n">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
@@ -6088,17 +6104,15 @@
         <v>20</v>
       </c>
       <c r="B72" s="18" t="n">
-        <v>234</v>
-      </c>
-      <c r="C72" s="19" t="inlineStr">
-        <is>
-          <t>Dawson Knox (TE BUF)</t>
-        </is>
-      </c>
-      <c r="D72" s="18" t="n">
-        <v>230.1</v>
-      </c>
-      <c r="E72" s="19" t="inlineStr"/>
+        <v>238</v>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>— no fit —</t>
+        </is>
+      </c>
+      <c r="D72" s="19" t="n"/>
+      <c r="E72" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6137,7 +6151,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 5 — Score 81</t>
+          <t>No Punt — Best slot 5 — Score 95</t>
         </is>
       </c>
     </row>
@@ -6543,7 +6557,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 7 — Score 78</t>
+          <t>R1 Punted — Best slot 7 — Score 91</t>
         </is>
       </c>
     </row>
@@ -6955,7 +6969,7 @@
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>R1-R2 Punted — Best slot 7 — Score 75</t>
+          <t>R1-R2 Punted — Best slot 7 — Score 88</t>
         </is>
       </c>
     </row>
@@ -7395,7 +7409,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 5 — Score 70</t>
+          <t>No Punt — Best slot 5 — Score 76</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7807,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 8 — Score 64</t>
+          <t>R1 Punted — Best slot 8 — Score 58</t>
         </is>
       </c>
     </row>
@@ -8189,7 +8203,7 @@
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>R1-R2 Punted — Best slot 8 — Score 64</t>
+          <t>R1-R2 Punted — Best slot 8 — Score 69</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8627,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 8 — Score 79</t>
+          <t>No Punt — Best slot 4 — Score 92</t>
         </is>
       </c>
     </row>
@@ -8649,7 +8663,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="18" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
@@ -8666,7 +8680,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
@@ -8687,19 +8701,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Breece Hall (RB NYJ)</t>
+          <t>Jeremiyah Love (RB ARI)</t>
         </is>
       </c>
       <c r="D7" s="18" t="n">
-        <v>33.8</v>
+        <v>25.9</v>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Garrett Wilson (38.6)</t>
+          <t>Breece Hall (33.8), Garrett Wilson (38.6)</t>
         </is>
       </c>
     </row>
@@ -8708,19 +8722,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="18" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Garrett Wilson (WR NYJ)</t>
+          <t>Jaylen Waddle (WR DEN)</t>
         </is>
       </c>
       <c r="D8" s="18" t="n">
-        <v>38.6</v>
+        <v>50</v>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Jaylen Waddle (50.0)</t>
+          <t>TreVeyon Henderson (56.3)</t>
         </is>
       </c>
     </row>
@@ -8729,7 +8743,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="18" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
@@ -8739,30 +8753,26 @@
       <c r="D9" s="18" t="n">
         <v>56.3</v>
       </c>
-      <c r="E9" s="19" t="inlineStr">
-        <is>
-          <t>Jaylen Waddle (50.0), Drake Maye (64.5), Marvin Harrison Jr. (65.5)</t>
-        </is>
-      </c>
+      <c r="E9" s="19" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="18" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="18" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Drake Maye (QB NE)</t>
+          <t>Marvin Harrison Jr. (WR ARI)</t>
         </is>
       </c>
       <c r="D10" s="18" t="n">
-        <v>64.5</v>
+        <v>65.5</v>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr. (65.5)</t>
+          <t>Drake Maye (64.5), RJ Harvey (77.2), Rhamondre Stevenson (78.9), Michael Wilson (80.4)</t>
         </is>
       </c>
     </row>
@@ -8771,19 +8781,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="18" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Michael Wilson (WR ARI)</t>
+          <t>RJ Harvey (RB DEN)</t>
         </is>
       </c>
       <c r="D11" s="18" t="n">
-        <v>80.40000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>RJ Harvey (77.2), Rhamondre Stevenson (78.9), Courtland Sutton (83.1)</t>
+          <t>Rhamondre Stevenson (78.9), Michael Wilson (80.4), Courtland Sutton (83.1)</t>
         </is>
       </c>
     </row>
@@ -8792,49 +8802,41 @@
         <v>8</v>
       </c>
       <c r="B12" s="18" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Courtland Sutton (WR DEN)</t>
+          <t>Bo Nix (QB DEN)</t>
         </is>
       </c>
       <c r="D12" s="18" t="n">
-        <v>83.09999999999999</v>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>Bo Nix (100.9)</t>
-        </is>
-      </c>
+        <v>100.9</v>
+      </c>
+      <c r="E12" s="19" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="18" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Bo Nix (QB DEN)</t>
+          <t>J.K. Dobbins (RB DEN)</t>
         </is>
       </c>
       <c r="D13" s="18" t="n">
-        <v>100.9</v>
-      </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>J.K. Dobbins (108.9), Romeo Doubs (112.4)</t>
-        </is>
-      </c>
+        <v>108.9</v>
+      </c>
+      <c r="E13" s="19" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="18" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="18" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
@@ -8844,18 +8846,14 @@
       <c r="D14" s="18" t="n">
         <v>112.4</v>
       </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>J.K. Dobbins (108.9)</t>
-        </is>
-      </c>
+      <c r="E14" s="19" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="18" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="18" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
@@ -8870,7 +8868,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="18" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
@@ -8880,26 +8878,30 @@
       <c r="D16" s="18" t="n">
         <v>142.1</v>
       </c>
-      <c r="E16" s="19" t="inlineStr"/>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Omar Cooper Jr. (149.4)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="18" t="n">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>Hunter Henry (TE NE)</t>
+          <t>Omar Cooper Jr. (WR NYJ)</t>
         </is>
       </c>
       <c r="D17" s="18" t="n">
-        <v>154.3</v>
+        <v>149.4</v>
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>Omar Cooper Jr. (149.4), Jacoby Brissett (156.8), Tyler Allgeier (157.3), Fernando Mendoza (159.8), Jalen Nailor (161.5)</t>
+          <t>Hunter Henry (154.3), Jacoby Brissett (156.8), Tyler Allgeier (157.3), Fernando Mendoza (159.8)</t>
         </is>
       </c>
     </row>
@@ -8908,19 +8910,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="18" t="n">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>Jalen Nailor (WR LV)</t>
+          <t>Tre Tucker (WR LV)</t>
         </is>
       </c>
       <c r="D18" s="18" t="n">
-        <v>161.5</v>
+        <v>166.4</v>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>Jacoby Brissett (156.8), Tyler Allgeier (157.3), Fernando Mendoza (159.8), Tre Tucker (166.4), Jonah Coleman (166.8), Geno Smith (168.1)</t>
+          <t>Fernando Mendoza (159.8), Jalen Nailor (161.5), Jonah Coleman (166.8), Geno Smith (168.1)</t>
         </is>
       </c>
     </row>
@@ -8929,24 +8931,28 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="n">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Mike Washington Jr. (RB LV)</t>
+          <t>Geno Smith (QB NYJ)</t>
         </is>
       </c>
       <c r="D19" s="18" t="n">
-        <v>185.7</v>
-      </c>
-      <c r="E19" s="19" t="inlineStr"/>
+        <v>168.1</v>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Jonah Coleman (166.8)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="n">
         <v>16</v>
       </c>
       <c r="B20" s="18" t="n">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
@@ -8956,14 +8962,18 @@
       <c r="D20" s="18" t="n">
         <v>191</v>
       </c>
-      <c r="E20" s="19" t="inlineStr"/>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Mike Washington Jr. (185.7), Braelon Allen (199.9)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="18" t="n">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
@@ -8984,19 +8994,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="18" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>Adonai Mitchell (WR NYJ)</t>
+          <t>Troy Franklin (WR DEN)</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>205.7</v>
+        <v>213.9</v>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>Troy Franklin (213.9)</t>
+          <t>Evan Engram (223.8)</t>
         </is>
       </c>
     </row>
@@ -9005,7 +9015,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="18" t="n">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
@@ -9026,7 +9036,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="18" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
@@ -9036,16 +9046,12 @@
       <c r="D24" s="18" t="n">
         <v>231.1</v>
       </c>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>Mason Taylor (229.8), Eli Raridon (230.3)</t>
-        </is>
-      </c>
+      <c r="E24" s="19" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 12 — Score 79</t>
+          <t>R1 Punted — Best slot 12 — Score 100</t>
         </is>
       </c>
     </row>
@@ -9467,7 +9473,7 @@
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>R1-R2 Punted — Best slot 8 — Score 74</t>
+          <t>R1-R2 Punted — Best slot 4 — Score 87</t>
         </is>
       </c>
     </row>
@@ -9503,7 +9509,7 @@
         <v>1</v>
       </c>
       <c r="B53" s="18" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C53" s="20" t="inlineStr">
         <is>
@@ -9518,7 +9524,7 @@
         <v>2</v>
       </c>
       <c r="B54" s="18" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C54" s="20" t="inlineStr">
         <is>
@@ -9533,19 +9539,19 @@
         <v>3</v>
       </c>
       <c r="B55" s="18" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Breece Hall (RB NYJ)</t>
+          <t>Jeremiyah Love (RB ARI)</t>
         </is>
       </c>
       <c r="D55" s="18" t="n">
-        <v>33.8</v>
+        <v>25.9</v>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>Garrett Wilson (38.6)</t>
+          <t>Breece Hall (33.8), Garrett Wilson (38.6)</t>
         </is>
       </c>
     </row>
@@ -9554,19 +9560,19 @@
         <v>4</v>
       </c>
       <c r="B56" s="18" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Garrett Wilson (WR NYJ)</t>
+          <t>Jaylen Waddle (WR DEN)</t>
         </is>
       </c>
       <c r="D56" s="18" t="n">
-        <v>38.6</v>
+        <v>50</v>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>Jaylen Waddle (50.0)</t>
+          <t>TreVeyon Henderson (56.3)</t>
         </is>
       </c>
     </row>
@@ -9575,7 +9581,7 @@
         <v>5</v>
       </c>
       <c r="B57" s="18" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
@@ -9585,30 +9591,26 @@
       <c r="D57" s="18" t="n">
         <v>56.3</v>
       </c>
-      <c r="E57" s="19" t="inlineStr">
-        <is>
-          <t>Jaylen Waddle (50.0), Drake Maye (64.5), Marvin Harrison Jr. (65.5)</t>
-        </is>
-      </c>
+      <c r="E57" s="19" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="18" t="n">
         <v>6</v>
       </c>
       <c r="B58" s="18" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Drake Maye (QB NE)</t>
+          <t>Marvin Harrison Jr. (WR ARI)</t>
         </is>
       </c>
       <c r="D58" s="18" t="n">
-        <v>64.5</v>
+        <v>65.5</v>
       </c>
       <c r="E58" s="19" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr. (65.5)</t>
+          <t>Drake Maye (64.5), RJ Harvey (77.2), Rhamondre Stevenson (78.9), Michael Wilson (80.4)</t>
         </is>
       </c>
     </row>
@@ -9617,19 +9619,19 @@
         <v>7</v>
       </c>
       <c r="B59" s="18" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Michael Wilson (WR ARI)</t>
+          <t>RJ Harvey (RB DEN)</t>
         </is>
       </c>
       <c r="D59" s="18" t="n">
-        <v>80.40000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t>RJ Harvey (77.2), Rhamondre Stevenson (78.9), Courtland Sutton (83.1)</t>
+          <t>Rhamondre Stevenson (78.9), Michael Wilson (80.4), Courtland Sutton (83.1)</t>
         </is>
       </c>
     </row>
@@ -9638,49 +9640,41 @@
         <v>8</v>
       </c>
       <c r="B60" s="18" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Courtland Sutton (WR DEN)</t>
+          <t>Bo Nix (QB DEN)</t>
         </is>
       </c>
       <c r="D60" s="18" t="n">
-        <v>83.09999999999999</v>
-      </c>
-      <c r="E60" s="19" t="inlineStr">
-        <is>
-          <t>Bo Nix (100.9)</t>
-        </is>
-      </c>
+        <v>100.9</v>
+      </c>
+      <c r="E60" s="19" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="18" t="n">
         <v>9</v>
       </c>
       <c r="B61" s="18" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Bo Nix (QB DEN)</t>
+          <t>J.K. Dobbins (RB DEN)</t>
         </is>
       </c>
       <c r="D61" s="18" t="n">
-        <v>100.9</v>
-      </c>
-      <c r="E61" s="19" t="inlineStr">
-        <is>
-          <t>J.K. Dobbins (108.9), Romeo Doubs (112.4)</t>
-        </is>
-      </c>
+        <v>108.9</v>
+      </c>
+      <c r="E61" s="19" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="18" t="n">
         <v>10</v>
       </c>
       <c r="B62" s="18" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
@@ -9690,18 +9684,14 @@
       <c r="D62" s="18" t="n">
         <v>112.4</v>
       </c>
-      <c r="E62" s="19" t="inlineStr">
-        <is>
-          <t>J.K. Dobbins (108.9)</t>
-        </is>
-      </c>
+      <c r="E62" s="19" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="18" t="n">
         <v>11</v>
       </c>
       <c r="B63" s="18" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C63" s="20" t="inlineStr">
         <is>
@@ -9716,7 +9706,7 @@
         <v>12</v>
       </c>
       <c r="B64" s="18" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
@@ -9726,26 +9716,30 @@
       <c r="D64" s="18" t="n">
         <v>142.1</v>
       </c>
-      <c r="E64" s="19" t="inlineStr"/>
+      <c r="E64" s="19" t="inlineStr">
+        <is>
+          <t>Omar Cooper Jr. (149.4)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="18" t="n">
         <v>13</v>
       </c>
       <c r="B65" s="18" t="n">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Hunter Henry (TE NE)</t>
+          <t>Omar Cooper Jr. (WR NYJ)</t>
         </is>
       </c>
       <c r="D65" s="18" t="n">
-        <v>154.3</v>
+        <v>149.4</v>
       </c>
       <c r="E65" s="19" t="inlineStr">
         <is>
-          <t>Omar Cooper Jr. (149.4), Jacoby Brissett (156.8), Tyler Allgeier (157.3), Fernando Mendoza (159.8), Jalen Nailor (161.5)</t>
+          <t>Hunter Henry (154.3), Jacoby Brissett (156.8), Tyler Allgeier (157.3), Fernando Mendoza (159.8)</t>
         </is>
       </c>
     </row>
@@ -9754,19 +9748,19 @@
         <v>14</v>
       </c>
       <c r="B66" s="18" t="n">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Jalen Nailor (WR LV)</t>
+          <t>Tre Tucker (WR LV)</t>
         </is>
       </c>
       <c r="D66" s="18" t="n">
-        <v>161.5</v>
+        <v>166.4</v>
       </c>
       <c r="E66" s="19" t="inlineStr">
         <is>
-          <t>Jacoby Brissett (156.8), Tyler Allgeier (157.3), Fernando Mendoza (159.8), Tre Tucker (166.4), Jonah Coleman (166.8), Geno Smith (168.1)</t>
+          <t>Fernando Mendoza (159.8), Jalen Nailor (161.5), Jonah Coleman (166.8), Geno Smith (168.1)</t>
         </is>
       </c>
     </row>
@@ -9775,24 +9769,28 @@
         <v>15</v>
       </c>
       <c r="B67" s="18" t="n">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Mike Washington Jr. (RB LV)</t>
+          <t>Geno Smith (QB NYJ)</t>
         </is>
       </c>
       <c r="D67" s="18" t="n">
-        <v>185.7</v>
-      </c>
-      <c r="E67" s="19" t="inlineStr"/>
+        <v>168.1</v>
+      </c>
+      <c r="E67" s="19" t="inlineStr">
+        <is>
+          <t>Jonah Coleman (166.8)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="18" t="n">
         <v>16</v>
       </c>
       <c r="B68" s="18" t="n">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
@@ -9802,14 +9800,18 @@
       <c r="D68" s="18" t="n">
         <v>191</v>
       </c>
-      <c r="E68" s="19" t="inlineStr"/>
+      <c r="E68" s="19" t="inlineStr">
+        <is>
+          <t>Mike Washington Jr. (185.7), Braelon Allen (199.9)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="18" t="n">
         <v>17</v>
       </c>
       <c r="B69" s="18" t="n">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
@@ -9830,19 +9832,19 @@
         <v>18</v>
       </c>
       <c r="B70" s="18" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Adonai Mitchell (WR NYJ)</t>
+          <t>Troy Franklin (WR DEN)</t>
         </is>
       </c>
       <c r="D70" s="18" t="n">
-        <v>205.7</v>
+        <v>213.9</v>
       </c>
       <c r="E70" s="19" t="inlineStr">
         <is>
-          <t>Troy Franklin (213.9)</t>
+          <t>Evan Engram (223.8)</t>
         </is>
       </c>
     </row>
@@ -9851,7 +9853,7 @@
         <v>19</v>
       </c>
       <c r="B71" s="18" t="n">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
@@ -9872,7 +9874,7 @@
         <v>20</v>
       </c>
       <c r="B72" s="18" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
@@ -9882,11 +9884,7 @@
       <c r="D72" s="18" t="n">
         <v>231.1</v>
       </c>
-      <c r="E72" s="19" t="inlineStr">
-        <is>
-          <t>Mason Taylor (229.8), Eli Raridon (230.3)</t>
-        </is>
-      </c>
+      <c r="E72" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -9925,7 +9923,7 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>No Punt — Best slot 5 — Score 74</t>
+          <t>No Punt — Best slot 5 — Score 80</t>
         </is>
       </c>
     </row>
@@ -10371,7 +10369,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>R1 Punted — Best slot 7 — Score 69</t>
+          <t>R1 Punted — Best slot 7 — Score 65</t>
         </is>
       </c>
     </row>
@@ -10815,7 +10813,7 @@
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>R1-R2 Punted — Best slot 7 — Score 70</t>
+          <t>R1-R2 Punted — Best slot 7 — Score 79</t>
         </is>
       </c>
     </row>

</xml_diff>